<commit_message>
feat: a supplier's filing frequency from the purchase register
An optional register column, "Supplier filing frequency" (Monthly or
Quarterly, any case; a few other titles accepted, and mappable), sets the
supplier's scheme as the trader's own: filing_scheme_source USER, the same as
PUT /api/suppliers/:gstin/filing-scheme, so whichever came last wins. A blank
cell says nothing; any other value is refused. The commit reports
filingSchemes { declared, changed }, and when a scheme changed every
reconciled period is re-run against the moved cut-off.

The demo registers say Krishna Enterprises files quarterly, so on 11 Sep
Krishna has 2 days left without a manual step. No contacts.local.json exists,
so fixtures/demo-local/ was not regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/demo/aug/purchase_register_aug26.xlsx
+++ b/fixtures/demo/aug/purchase_register_aug26.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:O16"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -414,6 +414,7 @@
     <col min="12" max="12" width="20.83203125" customWidth="1"/>
     <col min="13" max="13" width="17.83203125" customWidth="1"/>
     <col min="14" max="14" width="26.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,6 +488,9 @@
       <c r="N5" t="str">
         <v>Supplier email</v>
       </c>
+      <c r="O5" t="str">
+        <v>Supplier filing frequency</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -817,6 +821,9 @@
       <c r="N14" t="str">
         <v>supplier9@example.com</v>
       </c>
+      <c r="O14" t="str">
+        <v>Quarterly</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -893,7 +900,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>